<commit_message>
Add another ImagingStudy to the parameter example. Fix some confusion in the titles of the CS, VS and Extension. Comment and ignore more warnings and errors.
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-videre-forlop-cs.xlsx
+++ b/docs/CodeSystem-videre-forlop-cs.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Pending Grading Step</t>
+    <t>Grading Pending</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-12T18:21:01+01:00</t>
+    <t>2025-11-13T17:39:30+01:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Add code system grading-caution-cs (5000 series)
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-videre-forlop-cs.xlsx
+++ b/docs/CodeSystem-videre-forlop-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-15T17:14:08+01:00</t>
+    <t>2025-11-16T16:39:43+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -144,16 +144,25 @@
     <t>KI-gradering</t>
   </si>
   <si>
+    <t>Skal til KI-gradering.</t>
+  </si>
+  <si>
     <t>4002</t>
   </si>
   <si>
     <t>Primærgradering manuell</t>
   </si>
   <si>
+    <t>Fotograf har konkludert at bildene skal vurderes av en primærgraderer.</t>
+  </si>
+  <si>
     <t>4003</t>
   </si>
   <si>
     <t>Sekundærgradering manuell</t>
+  </si>
+  <si>
+    <t>Fotograf har konkludert at bildene skal vurderes av en sekundærgraderer.</t>
   </si>
 </sst>
 </file>
@@ -490,31 +499,37 @@
       <c r="C2" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" t="s" s="2">
+        <v>43</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
         <v>40</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>46</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
         <v>40</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D4" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>